<commit_message>
update staxi sáng 03/03/2026
</commit_message>
<xml_diff>
--- a/TAXI_ChecklistForAutoTestSTAXI.xlsx
+++ b/TAXI_ChecklistForAutoTestSTAXI.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13470"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="24000" windowHeight="10770"/>
   </bookViews>
   <sheets>
     <sheet name="Checklist" sheetId="1" r:id="rId1"/>
@@ -1365,7 +1365,7 @@
     <t>Hiển thị đúng Xe đã nhập ở danh sách và popup Hiện trạng</t>
   </si>
   <si>
-    <t>30E03710</t>
+    <t>30E03933</t>
   </si>
   <si>
     <t>Minitor68_.png</t>
@@ -3803,7 +3803,7 @@
     <t>Trường "Tên khuyến mại" hiện thị: Đúng "Tên" đã nhập</t>
   </si>
   <si>
-    <t>Auto_CaiAppMoi2318</t>
+    <t>KM cài app99900</t>
   </si>
   <si>
     <t>Promotion28</t>
@@ -7143,6 +7143,9 @@
 3. Tìm kiếm &gt; Check hiển thị</t>
   </si>
   <si>
+    <t>batrinh209a</t>
+  </si>
+  <si>
     <t>Report56</t>
   </si>
   <si>
@@ -7186,9 +7189,6 @@
   <si>
     <t>Có dữ liệu tìm kiếm hàng đầu tiên
 (Hiển thị )</t>
-  </si>
-  <si>
-    <t>batrinh209a</t>
   </si>
   <si>
     <t>Report59</t>
@@ -26106,8 +26106,8 @@
     <col min="13" max="13" width="20.42578125" style="21" customWidth="1"/>
     <col min="14" max="14" width="27.140625" style="21" customWidth="1"/>
     <col min="15" max="15" width="14.7109375" style="79" customWidth="1"/>
-    <col min="16" max="3152" width="9.140625" style="79" customWidth="1"/>
-    <col min="3153" max="16384" width="9.140625" style="79"/>
+    <col min="16" max="3163" width="9.140625" style="79" customWidth="1"/>
+    <col min="3164" max="16384" width="9.140625" style="79"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -41257,7 +41257,7 @@
         <v>1795</v>
       </c>
       <c r="F569" s="29" t="s">
-        <v>1748</v>
+        <v>1867</v>
       </c>
       <c r="G569" s="4" t="s">
         <v>4</v>
@@ -41274,14 +41274,14 @@
     </row>
     <row r="570" spans="1:14" ht="75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A570" s="37" t="s">
-        <v>1867</v>
+        <v>1868</v>
       </c>
       <c r="B570" s="37" t="s">
         <v>815</v>
       </c>
       <c r="C570" s="26"/>
       <c r="D570" s="15" t="s">
-        <v>1868</v>
+        <v>1869</v>
       </c>
       <c r="E570" s="15" t="s">
         <v>167</v>
@@ -41318,7 +41318,7 @@
     </row>
     <row r="572" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A572" s="49" t="s">
-        <v>1869</v>
+        <v>1870</v>
       </c>
       <c r="B572" s="49"/>
       <c r="C572" s="50" t="s">
@@ -41338,20 +41338,20 @@
     </row>
     <row r="573" spans="1:14" ht="56.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A573" s="37" t="s">
-        <v>1870</v>
+        <v>1871</v>
       </c>
       <c r="B573" s="39" t="s">
-        <v>1871</v>
+        <v>1872</v>
       </c>
       <c r="C573" s="26"/>
       <c r="D573" s="15" t="s">
-        <v>1872</v>
+        <v>1873</v>
       </c>
       <c r="E573" s="27" t="s">
-        <v>1873</v>
+        <v>1874</v>
       </c>
       <c r="F573" s="29" t="s">
-        <v>1874</v>
+        <v>1875</v>
       </c>
       <c r="G573" s="4" t="s">
         <v>4</v>
@@ -41368,20 +41368,20 @@
     </row>
     <row r="574" spans="1:14" ht="56.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A574" s="37" t="s">
-        <v>1875</v>
+        <v>1876</v>
       </c>
       <c r="B574" s="37" t="s">
         <v>1060</v>
       </c>
       <c r="C574" s="26"/>
       <c r="D574" s="29" t="s">
-        <v>1876</v>
+        <v>1877</v>
       </c>
       <c r="E574" s="29" t="s">
-        <v>1877</v>
+        <v>1878</v>
       </c>
       <c r="F574" s="29" t="s">
-        <v>1878</v>
+        <v>1867</v>
       </c>
       <c r="G574" s="4" t="s">
         <v>4</v>
@@ -41874,7 +41874,7 @@
         <v>1922</v>
       </c>
       <c r="E594" s="29" t="s">
-        <v>1877</v>
+        <v>1878</v>
       </c>
       <c r="F594" s="29"/>
       <c r="G594" s="4" t="s">
@@ -42000,10 +42000,10 @@
         <v>1932</v>
       </c>
       <c r="E599" s="29" t="s">
-        <v>1877</v>
+        <v>1878</v>
       </c>
       <c r="F599" s="29" t="s">
-        <v>1878</v>
+        <v>1867</v>
       </c>
       <c r="G599" s="4" t="s">
         <v>4</v>
@@ -42123,7 +42123,7 @@
         <v>1942</v>
       </c>
       <c r="E604" s="29" t="s">
-        <v>1877</v>
+        <v>1878</v>
       </c>
       <c r="F604" s="29" t="s">
         <v>1943</v>
@@ -42306,7 +42306,7 @@
         <v>1956</v>
       </c>
       <c r="E611" s="29" t="s">
-        <v>1877</v>
+        <v>1878</v>
       </c>
       <c r="F611" s="29" t="s">
         <v>1957</v>
@@ -47795,7 +47795,7 @@
         <v>2594</v>
       </c>
       <c r="E821" s="29" t="s">
-        <v>1877</v>
+        <v>1878</v>
       </c>
       <c r="F821" s="29" t="s">
         <v>2595</v>
@@ -47918,7 +47918,7 @@
         <v>2605</v>
       </c>
       <c r="E826" s="29" t="s">
-        <v>1877</v>
+        <v>1878</v>
       </c>
       <c r="F826" s="29" t="s">
         <v>2606</v>

</xml_diff>

<commit_message>
update staxi sáng 10/03/2026
</commit_message>
<xml_diff>
--- a/TAXI_ChecklistForAutoTestSTAXI.xlsx
+++ b/TAXI_ChecklistForAutoTestSTAXI.xlsx
@@ -15043,8 +15043,8 @@
     <col width="20.42578125" customWidth="1" style="21" min="13" max="13"/>
     <col width="27.140625" customWidth="1" style="21" min="14" max="14"/>
     <col width="14.7109375" customWidth="1" style="85" min="15" max="15"/>
-    <col width="9.140625" customWidth="1" style="85" min="16" max="3171"/>
-    <col width="9.140625" customWidth="1" style="85" min="3172" max="16384"/>
+    <col width="9.140625" customWidth="1" style="85" min="16" max="3176"/>
+    <col width="9.140625" customWidth="1" style="85" min="3177" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" customHeight="1">
@@ -15467,7 +15467,11 @@
           <t>x</t>
         </is>
       </c>
-      <c r="M12" s="20" t="n"/>
+      <c r="M12" s="20" t="inlineStr">
+        <is>
+          <t>Login01Login_Admin.png</t>
+        </is>
+      </c>
       <c r="N12" s="20" t="n"/>
     </row>
     <row r="13" ht="75" customHeight="1">
@@ -15522,7 +15526,11 @@
           <t>x</t>
         </is>
       </c>
-      <c r="M13" s="20" t="n"/>
+      <c r="M13" s="20" t="inlineStr">
+        <is>
+          <t>Login02Login_Admin.png</t>
+        </is>
+      </c>
       <c r="N13" s="20" t="n"/>
     </row>
     <row r="14" ht="75" customHeight="1">
@@ -15554,16 +15562,8 @@
 tài khoản: "Xin chào: [1996] Test 12/10 [1996]"</t>
         </is>
       </c>
-      <c r="F14" s="15" t="inlineStr">
-        <is>
-          <t>Xin chào: [1996] Test 12/10 [1996]</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
+      <c r="F14" s="15" t="n"/>
+      <c r="G14" s="4" t="n"/>
       <c r="H14" s="6" t="n"/>
       <c r="I14" s="6" t="n"/>
       <c r="J14" s="6" t="n"/>
@@ -16251,7 +16251,7 @@
       </c>
       <c r="F34" s="15" t="inlineStr">
         <is>
-          <t>26/2/2026</t>
+          <t>9/3/2026</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -16295,16 +16295,8 @@
           <t>Trường "Thời điểm mất kết nối" hiển thị dữ liệu hàng đầu tiên: "Ngày hiện tại"</t>
         </is>
       </c>
-      <c r="F35" s="15" t="inlineStr">
-        <is>
-          <t>26/2/2026</t>
-        </is>
-      </c>
-      <c r="G35" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
+      <c r="F35" s="15" t="n"/>
+      <c r="G35" s="4" t="n"/>
       <c r="H35" s="6" t="n"/>
       <c r="I35" s="6" t="n"/>
       <c r="J35" s="6" t="n"/>
@@ -16344,7 +16336,7 @@
       </c>
       <c r="F36" s="15" t="inlineStr">
         <is>
-          <t>Đóng</t>
+          <t>Mở</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -16390,10 +16382,14 @@
       </c>
       <c r="F37" s="15" t="inlineStr">
         <is>
-          <t>Không có dữ liệu</t>
-        </is>
-      </c>
-      <c r="G37" s="4" t="n"/>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="H37" s="6" t="n"/>
       <c r="I37" s="6" t="n"/>
       <c r="J37" s="6" t="n"/>
@@ -16436,14 +16432,10 @@
       </c>
       <c r="F38" s="15" t="inlineStr">
         <is>
-          <t>Đóng</t>
-        </is>
-      </c>
-      <c r="G38" s="4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
+          <t>Không có dữ liệu</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="n"/>
       <c r="H38" s="6" t="n"/>
       <c r="I38" s="6" t="n"/>
       <c r="J38" s="6" t="n"/>
@@ -16453,7 +16445,11 @@
         </is>
       </c>
       <c r="L38" s="4" t="n"/>
-      <c r="M38" s="20" t="n"/>
+      <c r="M38" s="20" t="inlineStr">
+        <is>
+          <t>Minitor09GiamSat_TimKiem_DangVaoCaVaMatKetNoi.png</t>
+        </is>
+      </c>
       <c r="N38" s="20" t="n"/>
     </row>
     <row r="39" ht="38.45" customHeight="1">
@@ -18885,8 +18881,8 @@
       </c>
       <c r="F98" s="15" t="inlineStr">
         <is>
-          <t>Biển số xe: Biển số xe: 18H04971
-Thời gian: Từ ngày: 25/02/2026 20:00 Đến ngày: 26/2/2026 19:22</t>
+          <t>Biển số xe: Biển số xe: 18H02826
+Thời gian: Từ ngày: 05/03/2026 20:00 Đến ngày: 6/3/2026 8:26</t>
         </is>
       </c>
       <c r="G98" s="4" t="inlineStr">

</xml_diff>